<commit_message>
Complete pilot PPR integration with scoped estimates and recycling views
Finish source-led pilot mappings and a new-paper pipeline validation, preserving
model identity, geographic limits and failed numerical configurations. Add
inner/PP workbooks, method ratios and GE/TE recycling controls, with coloring
restricted to selected pilot ecosystems.

Rebuild and verify the ecosystem and upstream exports, preserve missing values
and correct the wet-weight/carbon comparison. Keep equivalent Claude and Codex
skill sets and refresh the knowledge graph for the completed integration.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PPREstimation/output/top10/13_2_Northern_Humboldt_Current_(1995-1998).xlsx
+++ b/PPREstimation/output/top10/13_2_Northern_Humboldt_Current_(1995-1998).xlsx
@@ -701,7 +701,11 @@
           <t>DET</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Non-consuming egg/detritus or external input pool; no catch assignment.</t>
+        </is>
+      </c>
       <c r="F3" s="2" t="n">
         <v>1</v>
       </c>
@@ -785,7 +789,11 @@
           <t>DET</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Non-consuming egg/detritus or external input pool; no catch assignment.</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="n">
         <v>1</v>
       </c>
@@ -869,7 +877,11 @@
           <t>DET</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Non-consuming egg/detritus or external input pool; no catch assignment.</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="n">
         <v>1</v>
       </c>
@@ -953,7 +965,11 @@
           <t>DET</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Non-consuming egg/detritus or external input pool; no catch assignment.</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="n">
         <v>1</v>
       </c>
@@ -1037,7 +1053,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Dermochelys coriacea; definition: Named taxon; source spellings and verified aliases retained in members.csv.</t>
+        </is>
+      </c>
       <c r="F7" s="2" t="n">
         <v>4.036651412301057</v>
       </c>
@@ -1121,7 +1141,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Chelonia mydas; definition: Named taxon; source spellings and verified aliases retained in members.csv.</t>
+        </is>
+      </c>
       <c r="F8" s="2" t="n">
         <v>3.483659556323609</v>
       </c>
@@ -1205,7 +1229,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Cetaceans; no species list documented.</t>
+        </is>
+      </c>
       <c r="F9" s="2" t="n">
         <v>4.211135921072626</v>
       </c>
@@ -1289,7 +1317,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Otaria flavescens; Arctocephalus australis; definition: not documented - no species list found for this source group.</t>
+        </is>
+      </c>
       <c r="F10" s="2" t="n">
         <v>3.748751632707471</v>
       </c>
@@ -1373,7 +1405,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Phalacrocorax bougainvillii; Sula variegata; Pelecanus thagus; definition: not documented - no species list found for this source group.</t>
+        </is>
+      </c>
       <c r="F11" s="2" t="n">
         <v>3.92938764796025</v>
       </c>
@@ -1457,7 +1493,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Chondrichthyans other than the separately modelled benthic elasmobranch pool; Table E aggregates as apex predatory fish.</t>
+        </is>
+      </c>
       <c r="F12" s="2" t="n">
         <v>4.559153783576394</v>
       </c>
@@ -1541,7 +1581,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Galeichtys peruvianus; definition: Named taxon; source spellings and verified aliases retained in members.csv.</t>
+        </is>
+      </c>
       <c r="F13" s="2" t="n">
         <v>3.148778445321641</v>
       </c>
@@ -1625,7 +1669,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Prionotus stephanophrys; definition: Named taxon; source spellings and verified aliases retained in members.csv.</t>
+        </is>
+      </c>
       <c r="F14" s="2" t="n">
         <v>3.329151265268742</v>
       </c>
@@ -1709,7 +1757,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Medium sciaenids; no full species list documented. Ctenosciaena peruviana is explicitly in Small demersal fish. Table E aggregates as demersal benthivorous fish.</t>
+        </is>
+      </c>
       <c r="F15" s="2" t="n">
         <v>3.376461817236302</v>
       </c>
@@ -1793,7 +1845,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Paralabrax humeralis; Hemanthias peruanus; Mugil cephalus; definition: Medium demersal fishes, source examples Paralabrax, Hemanthias and Mugil; Table E aggregates as demersal benthivorous fish.</t>
+        </is>
+      </c>
       <c r="F16" s="2" t="n">
         <v>3.2413623234645</v>
       </c>
@@ -1877,7 +1933,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Congers; no species list documented. Table E aggregates as demersal piscivorous fish.</t>
+        </is>
+      </c>
       <c r="F17" s="2" t="n">
         <v>4.165306519244008</v>
       </c>
@@ -1961,7 +2021,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Trachinotus paitensis; Stromateus stellatus; Peprilus medius; definition: Butter fishes; named examples Trachinotus, Stromateus and Peprilus. Table E aggregates as pelagic planktivorous fish.</t>
+        </is>
+      </c>
       <c r="F18" s="2" t="n">
         <v>2.633052892562976</v>
       </c>
@@ -2045,7 +2109,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Benthic elasmobranchs, separate from Chondrichthyans; Table E aggregates as demersal benthivorous fish.</t>
+        </is>
+      </c>
       <c r="F19" s="2" t="n">
         <v>3.404504687960284</v>
       </c>
@@ -2129,7 +2197,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Odonthestes regia; Labrisomus philippi; Ctenosciaena peruviana; definition: Small demersal fishes; source examples take precedence over habitat heuristics. Table E aggregates as demersal planktivorous fish.</t>
+        </is>
+      </c>
       <c r="F20" s="2" t="n">
         <v>2.472727272727273</v>
       </c>
@@ -2213,7 +2285,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Paralichthys adspersus; Hippoglosina sp.; definition: Flatfishes; Table E aggregates as demersal piscivorous fish.</t>
+        </is>
+      </c>
       <c r="F21" s="2" t="n">
         <v>3.92129953038265</v>
       </c>
@@ -2297,7 +2373,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>M. gayi peruanus; definition: Peruvian hake Merluccius gayi peruanus, &gt;50 cm. Printed interval endpoints retained; catch is unaged.</t>
+        </is>
+      </c>
       <c r="F22" s="2" t="n">
         <v>4.376603472176864</v>
       </c>
@@ -2381,7 +2461,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>M. gayi peruanus; definition: Peruvian hake Merluccius gayi peruanus, 30-49 cm. Printed interval endpoints retained; catch is unaged.</t>
+        </is>
+      </c>
       <c r="F23" s="2" t="n">
         <v>3.867970436464992</v>
       </c>
@@ -2465,7 +2549,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Merluccius gayi peruanus; definition: Peruvian hake Merluccius gayi peruanus, &lt;29 cm. Printed interval endpoints retained; catch is unaged.</t>
+        </is>
+      </c>
       <c r="F24" s="2" t="n">
         <v>3.730402926500451</v>
       </c>
@@ -2549,7 +2637,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Sarda chiliensis; Coryphaena hippurus; Thunnus albacares; definition: Other large pelagic fishes; source examples are bonito, dolphinfish and yellowfin tuna. Table E calls the aggregate pelagic piscivorous fish.</t>
+        </is>
+      </c>
       <c r="F25" s="2" t="n">
         <v>3.897127954782604</v>
       </c>
@@ -2633,7 +2725,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Scomber japonicus; definition: Named taxon; source spellings and verified aliases retained in members.csv.</t>
+        </is>
+      </c>
       <c r="F26" s="2" t="n">
         <v>3.601955384262967</v>
       </c>
@@ -2717,7 +2813,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Trachurus murphyi; definition: Named taxon; source spellings and verified aliases retained in members.csv.</t>
+        </is>
+      </c>
       <c r="F27" s="2" t="n">
         <v>3.445340771821614</v>
       </c>
@@ -2801,7 +2901,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Anchoa nasus; definition: Other small pelagic fish, excluding anchovy and sardine; Table E aggregates them as pelagic planktivorous fish.</t>
+        </is>
+      </c>
       <c r="F28" s="2" t="n">
         <v>2.768181818181818</v>
       </c>
@@ -2885,7 +2989,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Loligo gahi; Octopus vulgaris; Logigunculla sp.; definition: Cephalopods other than the separately modelled jumbo squid Dosidicus gigas.</t>
+        </is>
+      </c>
       <c r="F29" s="2" t="n">
         <v>3.174424242424243</v>
       </c>
@@ -2969,7 +3077,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Dosidicus gigas; definition: Named taxon; source spellings and verified aliases retained in members.csv.</t>
+        </is>
+      </c>
       <c r="F30" s="2" t="n">
         <v>4.086797321850294</v>
       </c>
@@ -3053,7 +3165,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Vinciguerria lucetia; Lampanyctus spp.; Leuroglossus spp.; definition: Mesopelagic fishes; species/genus examples in Tam (2008) section 2.1.</t>
+        </is>
+      </c>
       <c r="F31" s="2" t="n">
         <v>3.284848484848485</v>
       </c>
@@ -3137,7 +3253,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Engraulis ringens; definition: Named taxon; source spellings and verified aliases retained in members.csv.</t>
+        </is>
+      </c>
       <c r="F32" s="2" t="n">
         <v>2.934081345765596</v>
       </c>
@@ -3221,7 +3341,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Sardinops sagax; definition: Named taxon; source spellings and verified aliases retained in members.csv.</t>
+        </is>
+      </c>
       <c r="F33" s="2" t="n">
         <v>3.081475158660141</v>
       </c>
@@ -3305,7 +3429,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Benthic macroinvertebrates; no species membership list documented in focal paper, supplement or Tam predecessor.</t>
+        </is>
+      </c>
       <c r="F34" s="2" t="n">
         <v>2.052631578947368</v>
       </c>
@@ -3389,7 +3517,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Chrysaora plocamia; definition: Named taxon; source spellings and verified aliases retained in members.csv.</t>
+        </is>
+      </c>
       <c r="F35" s="2" t="n">
         <v>3.051393802259995</v>
       </c>
@@ -3473,7 +3605,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Small gelatinous zooplankton; Chrysaora plocamia is excluded into its own focal-model group.</t>
+        </is>
+      </c>
       <c r="F36" s="2" t="n">
         <v>2.992424242424243</v>
       </c>
@@ -3557,7 +3693,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Macrozooplankton 2-20 mm.</t>
+        </is>
+      </c>
       <c r="F37" s="2" t="n">
         <v>2.303030303030303</v>
       </c>
@@ -3641,7 +3781,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Mesozooplankton 200-2000 micrometres.</t>
+        </is>
+      </c>
       <c r="F38" s="2" t="n">
         <v>2.181818181818182</v>
       </c>
@@ -3725,7 +3869,11 @@
           <t>Regular</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Microzooplankton 20-200 micrometres.</t>
+        </is>
+      </c>
       <c r="F39" s="2" t="n">
         <v>2.212121212121212</v>
       </c>
@@ -3809,7 +3957,11 @@
           <t>PP</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Dinoflagellates and silicoflagellates.</t>
+        </is>
+      </c>
       <c r="F40" s="2" t="n">
         <v>1</v>
       </c>
@@ -3893,7 +4045,11 @@
           <t>PP</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Diatoms.</t>
+        </is>
+      </c>
       <c r="F41" s="2" t="n">
         <v>1</v>
       </c>
@@ -4159,7 +4315,9 @@
         <v>0</v>
       </c>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V2" s="2" t="n">
         <v>0</v>
       </c>
@@ -4217,7 +4375,9 @@
       <c r="T3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V3" s="2" t="n">
         <v>0</v>
       </c>
@@ -4275,7 +4435,9 @@
       <c r="T4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V4" s="2" t="n">
         <v>0</v>
       </c>
@@ -4333,7 +4495,9 @@
       <c r="T5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="U5" t="inlineStr"/>
+      <c r="U5" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V5" s="2" t="n">
         <v>0</v>
       </c>
@@ -4391,7 +4555,9 @@
       <c r="T6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V6" s="2" t="n">
         <v>0</v>
       </c>
@@ -4447,7 +4613,9 @@
       <c r="T7" s="2" t="n">
         <v>93.3598933783363</v>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" s="2" t="n">
+        <v>329.8300526420346</v>
+      </c>
       <c r="V7" s="2" t="n">
         <v>0</v>
       </c>
@@ -4503,7 +4671,9 @@
       <c r="T8" s="2" t="n">
         <v>38.9436369955784</v>
       </c>
-      <c r="U8" t="inlineStr"/>
+      <c r="U8" s="2" t="n">
+        <v>130.9805801156029</v>
+      </c>
       <c r="V8" s="2" t="n">
         <v>0</v>
       </c>
@@ -4559,7 +4729,9 @@
       <c r="T9" s="2" t="n">
         <v>4662.88804608467</v>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" s="2" t="n">
+        <v>15062.69347503343</v>
+      </c>
       <c r="V9" s="2" t="n">
         <v>0</v>
       </c>
@@ -4615,7 +4787,9 @@
       <c r="T10" s="2" t="n">
         <v>2978.011516236098</v>
       </c>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" s="2" t="n">
+        <v>7852.979598968306</v>
+      </c>
       <c r="V10" s="2" t="n">
         <v>0</v>
       </c>
@@ -4671,7 +4845,9 @@
       <c r="T11" s="2" t="n">
         <v>14683.24346635239</v>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" s="2" t="n">
+        <v>40258.57746310868</v>
+      </c>
       <c r="V11" s="2" t="n">
         <v>0</v>
       </c>
@@ -4729,9 +4905,11 @@
       <c r="T12" s="2" t="n">
         <v>195.2023859866585</v>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" s="2" t="n">
+        <v>628.5731936635907</v>
+      </c>
       <c r="V12" s="2" t="n">
-        <v>8719.621807822547</v>
+        <v>9364.462679720415</v>
       </c>
     </row>
     <row r="13">
@@ -4787,9 +4965,11 @@
       <c r="T13" s="2" t="n">
         <v>8.15664640193301</v>
       </c>
-      <c r="U13" t="inlineStr"/>
+      <c r="U13" s="2" t="n">
+        <v>20.74595787825953</v>
+      </c>
       <c r="V13" s="2" t="n">
-        <v>58.7795138381428</v>
+        <v>57.97407860326917</v>
       </c>
     </row>
     <row r="14">
@@ -4845,9 +5025,11 @@
       <c r="T14" s="2" t="n">
         <v>14.80448689328681</v>
       </c>
-      <c r="U14" t="inlineStr"/>
+      <c r="U14" s="2" t="n">
+        <v>26.42535486733363</v>
+      </c>
       <c r="V14" s="2" t="n">
-        <v>120.6555955779325</v>
+        <v>122.7283630538291</v>
       </c>
     </row>
     <row r="15">
@@ -4903,9 +5085,11 @@
       <c r="T15" s="2" t="n">
         <v>26.89192646900239</v>
       </c>
-      <c r="U15" t="inlineStr"/>
+      <c r="U15" s="2" t="n">
+        <v>76.47780119191297</v>
+      </c>
       <c r="V15" s="2" t="n">
-        <v>5715.242438747673</v>
+        <v>5849.300316241179</v>
       </c>
     </row>
     <row r="16">
@@ -4961,9 +5145,11 @@
       <c r="T16" s="2" t="n">
         <v>13.49617829135049</v>
       </c>
-      <c r="U16" t="inlineStr"/>
+      <c r="U16" s="2" t="n">
+        <v>28.27997620255626</v>
+      </c>
       <c r="V16" s="2" t="n">
-        <v>79.53245924078773</v>
+        <v>76.95169782704731</v>
       </c>
     </row>
     <row r="17">
@@ -5019,9 +5205,11 @@
       <c r="T17" s="2" t="n">
         <v>119.1536398888879</v>
       </c>
-      <c r="U17" t="inlineStr"/>
+      <c r="U17" s="2" t="n">
+        <v>352.8688649082416</v>
+      </c>
       <c r="V17" s="2" t="n">
-        <v>491634.4391305646</v>
+        <v>518378.2638005203</v>
       </c>
     </row>
     <row r="18">
@@ -5077,9 +5265,11 @@
       <c r="T18" s="2" t="n">
         <v>4.77521568509442</v>
       </c>
-      <c r="U18" t="inlineStr"/>
+      <c r="U18" s="2" t="n">
+        <v>12.26305011410535</v>
+      </c>
       <c r="V18" s="2" t="n">
-        <v>365799.4279695387</v>
+        <v>368049.7117824112</v>
       </c>
     </row>
     <row r="19">
@@ -5135,9 +5325,11 @@
       <c r="T19" s="2" t="n">
         <v>32.74580900913016</v>
       </c>
-      <c r="U19" t="inlineStr"/>
+      <c r="U19" s="2" t="n">
+        <v>88.50426598936681</v>
+      </c>
       <c r="V19" s="2" t="n">
-        <v>9041.886632940366</v>
+        <v>9306.463403563965</v>
       </c>
     </row>
     <row r="20">
@@ -5193,9 +5385,11 @@
       <c r="T20" s="2" t="n">
         <v>8.77424187851827</v>
       </c>
-      <c r="U20" t="inlineStr"/>
+      <c r="U20" s="2" t="n">
+        <v>15.20910093043284</v>
+      </c>
       <c r="V20" s="2" t="n">
-        <v>30.61949382134773</v>
+        <v>30.24186607511134</v>
       </c>
     </row>
     <row r="21">
@@ -5251,9 +5445,11 @@
       <c r="T21" s="2" t="n">
         <v>55.9614934730272</v>
       </c>
-      <c r="U21" t="inlineStr"/>
+      <c r="U21" s="2" t="n">
+        <v>167.6292882553963</v>
+      </c>
       <c r="V21" s="2" t="n">
-        <v>358.4885016531974</v>
+        <v>355.9925753030737</v>
       </c>
     </row>
     <row r="22">
@@ -5309,9 +5505,11 @@
       <c r="T22" s="2" t="n">
         <v>156.8641762627951</v>
       </c>
-      <c r="U22" t="inlineStr"/>
+      <c r="U22" s="2" t="n">
+        <v>599.1192070707298</v>
+      </c>
       <c r="V22" s="2" t="n">
-        <v>54263.25630566836</v>
+        <v>54468.06839372768</v>
       </c>
     </row>
     <row r="23">
@@ -5367,9 +5565,11 @@
       <c r="T23" s="2" t="n">
         <v>62.6185180135832</v>
       </c>
-      <c r="U23" t="inlineStr"/>
+      <c r="U23" s="2" t="n">
+        <v>148.9674428802408</v>
+      </c>
       <c r="V23" s="2" t="n">
-        <v>3599.433765358843</v>
+        <v>3756.974335796574</v>
       </c>
     </row>
     <row r="24">
@@ -5425,9 +5625,11 @@
       <c r="T24" s="2" t="n">
         <v>42.0271777140439</v>
       </c>
-      <c r="U24" t="inlineStr"/>
+      <c r="U24" s="2" t="n">
+        <v>133.1718490436824</v>
+      </c>
       <c r="V24" s="2" t="n">
-        <v>870.5705143647886</v>
+        <v>873.4544605300705</v>
       </c>
     </row>
     <row r="25">
@@ -5483,9 +5685,11 @@
       <c r="T25" s="2" t="n">
         <v>93.36028271793721</v>
       </c>
-      <c r="U25" t="inlineStr"/>
+      <c r="U25" s="2" t="n">
+        <v>238.4009240486365</v>
+      </c>
       <c r="V25" s="2" t="n">
-        <v>1466.805513860761</v>
+        <v>1534.363238304007</v>
       </c>
     </row>
     <row r="26">
@@ -5541,9 +5745,11 @@
       <c r="T26" s="2" t="n">
         <v>64.490704399306</v>
       </c>
-      <c r="U26" t="inlineStr"/>
+      <c r="U26" s="2" t="n">
+        <v>167.5412765408897</v>
+      </c>
       <c r="V26" s="2" t="n">
-        <v>2241.303470499185</v>
+        <v>2202.672861758966</v>
       </c>
     </row>
     <row r="27">
@@ -5599,9 +5805,11 @@
       <c r="T27" s="2" t="n">
         <v>35.0656057045034</v>
       </c>
-      <c r="U27" t="inlineStr"/>
+      <c r="U27" s="2" t="n">
+        <v>98.54234323175997</v>
+      </c>
       <c r="V27" s="2" t="n">
-        <v>914.7471558289719</v>
+        <v>912.4969484235231</v>
       </c>
     </row>
     <row r="28">
@@ -5657,9 +5865,11 @@
       <c r="T28" s="2" t="n">
         <v>12.98961292613629</v>
       </c>
-      <c r="U28" t="inlineStr"/>
+      <c r="U28" s="2" t="n">
+        <v>31.31069154482918</v>
+      </c>
       <c r="V28" s="2" t="n">
-        <v>51.47680407947213</v>
+        <v>52.04538846348984</v>
       </c>
     </row>
     <row r="29">
@@ -5715,9 +5925,11 @@
       <c r="T29" s="2" t="n">
         <v>4.9360974180695</v>
       </c>
-      <c r="U29" t="inlineStr"/>
+      <c r="U29" s="2" t="n">
+        <v>7.630091079247528</v>
+      </c>
       <c r="V29" s="2" t="n">
-        <v>15.84363644687813</v>
+        <v>15.74045856603944</v>
       </c>
     </row>
     <row r="30">
@@ -5773,9 +5985,11 @@
       <c r="T30" s="2" t="n">
         <v>36.2010618156066</v>
       </c>
-      <c r="U30" t="inlineStr"/>
+      <c r="U30" s="2" t="n">
+        <v>102.1369852454005</v>
+      </c>
       <c r="V30" s="2" t="n">
-        <v>973.8168227278527</v>
+        <v>1052.784035982254</v>
       </c>
     </row>
     <row r="31">
@@ -5831,9 +6045,11 @@
       <c r="T31" s="2" t="n">
         <v>18.47332305895662</v>
       </c>
-      <c r="U31" t="inlineStr"/>
+      <c r="U31" s="2" t="n">
+        <v>36.84655324199916</v>
+      </c>
       <c r="V31" s="2" t="n">
-        <v>257.2314406079555</v>
+        <v>264.6352371056698</v>
       </c>
     </row>
     <row r="32">
@@ -5889,9 +6105,11 @@
       <c r="T32" s="2" t="n">
         <v>11.26831373991057</v>
       </c>
-      <c r="U32" t="inlineStr"/>
+      <c r="U32" s="2" t="n">
+        <v>23.33269092207058</v>
+      </c>
       <c r="V32" s="2" t="n">
-        <v>49.44234709626252</v>
+        <v>49.22352449576737</v>
       </c>
     </row>
     <row r="33">
@@ -5947,9 +6165,11 @@
       <c r="T33" s="2" t="n">
         <v>13.95820929634474</v>
       </c>
-      <c r="U33" t="inlineStr"/>
+      <c r="U33" s="2" t="n">
+        <v>30.61064370997191</v>
+      </c>
       <c r="V33" s="2" t="n">
-        <v>55.21649223390927</v>
+        <v>54.37521282713333</v>
       </c>
     </row>
     <row r="34">
@@ -6005,7 +6225,9 @@
       <c r="T34" s="2" t="n">
         <v>-4.16928100533256e-14</v>
       </c>
-      <c r="U34" t="inlineStr"/>
+      <c r="U34" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V34" s="2" t="n">
         <v>0</v>
       </c>
@@ -6063,9 +6285,11 @@
       <c r="T35" s="2" t="n">
         <v>6.02271404967469</v>
       </c>
-      <c r="U35" t="inlineStr"/>
+      <c r="U35" s="2" t="n">
+        <v>16.75589838390295</v>
+      </c>
       <c r="V35" s="2" t="n">
-        <v>434511.4558208574</v>
+        <v>432377.2805293642</v>
       </c>
     </row>
     <row r="36">
@@ -6121,9 +6345,11 @@
       <c r="T36" s="2" t="n">
         <v>7.53914311447836</v>
       </c>
-      <c r="U36" t="inlineStr"/>
+      <c r="U36" s="2" t="n">
+        <v>18.96114406377533</v>
+      </c>
       <c r="V36" s="2" t="n">
-        <v>34.58797955858259</v>
+        <v>34.44567748145593</v>
       </c>
     </row>
     <row r="37">
@@ -6179,9 +6405,11 @@
       <c r="T37" s="2" t="n">
         <v>2.882483214733592</v>
       </c>
-      <c r="U37" t="inlineStr"/>
+      <c r="U37" s="2" t="n">
+        <v>3.486710728595533</v>
+      </c>
       <c r="V37" s="2" t="n">
-        <v>6.806530774155014</v>
+        <v>6.798716360355339</v>
       </c>
     </row>
     <row r="38">
@@ -6237,9 +6465,11 @@
       <c r="T38" s="2" t="n">
         <v>2.612926136363628</v>
       </c>
-      <c r="U38" t="inlineStr"/>
+      <c r="U38" s="2" t="n">
+        <v>4.040013778726465</v>
+      </c>
       <c r="V38" s="2" t="n">
-        <v>6.748256808111043</v>
+        <v>6.701891479903765</v>
       </c>
     </row>
     <row r="39">
@@ -6295,9 +6525,11 @@
       <c r="T39" s="2" t="n">
         <v>2.909090909090905</v>
       </c>
-      <c r="U39" t="inlineStr"/>
+      <c r="U39" s="2" t="n">
+        <v>3.255879985173817</v>
+      </c>
       <c r="V39" s="2" t="n">
-        <v>7.614973097363993</v>
+        <v>7.435466290384134</v>
       </c>
     </row>
     <row r="40">
@@ -6353,7 +6585,9 @@
       <c r="T40" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="U40" t="inlineStr"/>
+      <c r="U40" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V40" s="2" t="n">
         <v>1</v>
       </c>
@@ -6411,7 +6645,9 @@
       <c r="T41" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="U41" t="inlineStr"/>
+      <c r="U41" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V41" s="2" t="n">
         <v>1</v>
       </c>
@@ -6623,7 +6859,9 @@
         <v>0</v>
       </c>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V2" s="2" t="n">
         <v>0</v>
       </c>
@@ -6687,7 +6925,9 @@
       <c r="T3" s="2" t="n">
         <v>11.45573268643595</v>
       </c>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" s="2" t="n">
+        <v>96.79725031481013</v>
+      </c>
       <c r="V3" s="2" t="n">
         <v>0</v>
       </c>
@@ -6751,9 +6991,11 @@
       <c r="T4" s="2" t="n">
         <v>11.45573268643596</v>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" s="2" t="n">
+        <v>31.99787761378754</v>
+      </c>
       <c r="V4" s="2" t="n">
-        <v>0.3042852088602726</v>
+        <v>0.3042852088602723</v>
       </c>
     </row>
     <row r="5">
@@ -6815,7 +7057,9 @@
       <c r="T5" s="2" t="n">
         <v>11.45573268643596</v>
       </c>
-      <c r="U5" t="inlineStr"/>
+      <c r="U5" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V5" s="2" t="n">
         <v>0</v>
       </c>
@@ -6879,7 +7123,9 @@
       <c r="T6" s="2" t="n">
         <v>11.455732686436</v>
       </c>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" s="2" t="n">
+        <v>70.93194274175305</v>
+      </c>
       <c r="V6" s="2" t="n">
         <v>0</v>
       </c>
@@ -6943,7 +7189,9 @@
       <c r="T7" s="2" t="n">
         <v>589.4330104532831</v>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" s="2" t="n">
+        <v>16768.7649463136</v>
+      </c>
       <c r="V7" s="2" t="n">
         <v>0</v>
       </c>
@@ -7007,7 +7255,9 @@
       <c r="T8" s="2" t="n">
         <v>980.7365113181207</v>
       </c>
-      <c r="U8" t="inlineStr"/>
+      <c r="U8" s="2" t="n">
+        <v>16121.77397378537</v>
+      </c>
       <c r="V8" s="2" t="n">
         <v>0</v>
       </c>
@@ -7071,7 +7321,9 @@
       <c r="T9" s="2" t="n">
         <v>28180.96214906132</v>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" s="2" t="n">
+        <v>738053.459371696</v>
+      </c>
       <c r="V9" s="2" t="n">
         <v>0</v>
       </c>
@@ -7135,7 +7387,9 @@
       <c r="T10" s="2" t="n">
         <v>17085.22524944139</v>
       </c>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" s="2" t="n">
+        <v>336287.4499471319</v>
+      </c>
       <c r="V10" s="2" t="n">
         <v>0</v>
       </c>
@@ -7199,7 +7453,9 @@
       <c r="T11" s="2" t="n">
         <v>79503.20618141702</v>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" s="2" t="n">
+        <v>1740473.670358903</v>
+      </c>
       <c r="V11" s="2" t="n">
         <v>0</v>
       </c>
@@ -7263,9 +7519,11 @@
       <c r="T12" s="2" t="n">
         <v>1204.974224328892</v>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" s="2" t="n">
+        <v>32225.77357871431</v>
+      </c>
       <c r="V12" s="2" t="n">
-        <v>8719.621807822547</v>
+        <v>9364.462679720415</v>
       </c>
     </row>
     <row r="13">
@@ -7327,9 +7585,11 @@
       <c r="T13" s="2" t="n">
         <v>513.2343895775091</v>
       </c>
-      <c r="U13" t="inlineStr"/>
+      <c r="U13" s="2" t="n">
+        <v>6525.407273657614</v>
+      </c>
       <c r="V13" s="2" t="n">
-        <v>58.7795138381428</v>
+        <v>57.97407860326917</v>
       </c>
     </row>
     <row r="14">
@@ -7391,9 +7651,11 @@
       <c r="T14" s="2" t="n">
         <v>126.3294177567451</v>
       </c>
-      <c r="U14" t="inlineStr"/>
+      <c r="U14" s="2" t="n">
+        <v>1663.634074822245</v>
+      </c>
       <c r="V14" s="2" t="n">
-        <v>120.6555955779325</v>
+        <v>122.7283630538291</v>
       </c>
     </row>
     <row r="15">
@@ -7455,9 +7717,11 @@
       <c r="T15" s="2" t="n">
         <v>467.1943300954471</v>
       </c>
-      <c r="U15" t="inlineStr"/>
+      <c r="U15" s="2" t="n">
+        <v>8372.087825950925</v>
+      </c>
       <c r="V15" s="2" t="n">
-        <v>5715.242438747673</v>
+        <v>5849.300316241179</v>
       </c>
     </row>
     <row r="16">
@@ -7519,9 +7783,11 @@
       <c r="T16" s="2" t="n">
         <v>411.5163744177383</v>
       </c>
-      <c r="U16" t="inlineStr"/>
+      <c r="U16" s="2" t="n">
+        <v>4936.646120944995</v>
+      </c>
       <c r="V16" s="2" t="n">
-        <v>79.53245924078773</v>
+        <v>76.95169782704731</v>
       </c>
     </row>
     <row r="17">
@@ -7583,9 +7849,11 @@
       <c r="T17" s="2" t="n">
         <v>1438.417912447886</v>
       </c>
-      <c r="U17" t="inlineStr"/>
+      <c r="U17" s="2" t="n">
+        <v>28202.91345216605</v>
+      </c>
       <c r="V17" s="2" t="n">
-        <v>491634.4391305646</v>
+        <v>518378.2638005203</v>
       </c>
     </row>
     <row r="18">
@@ -7647,9 +7915,11 @@
       <c r="T18" s="2" t="n">
         <v>144.8466506925902</v>
       </c>
-      <c r="U18" t="inlineStr"/>
+      <c r="U18" s="2" t="n">
+        <v>2135.61323675179</v>
+      </c>
       <c r="V18" s="2" t="n">
-        <v>365799.4279695387</v>
+        <v>368049.7117824112</v>
       </c>
     </row>
     <row r="19">
@@ -7711,9 +7981,11 @@
       <c r="T19" s="2" t="n">
         <v>574.3013206749507</v>
       </c>
-      <c r="U19" t="inlineStr"/>
+      <c r="U19" s="2" t="n">
+        <v>8947.059362770606</v>
+      </c>
       <c r="V19" s="2" t="n">
-        <v>9041.886632940366</v>
+        <v>9306.463403563965</v>
       </c>
     </row>
     <row r="20">
@@ -7775,9 +8047,11 @@
       <c r="T20" s="2" t="n">
         <v>31.78984884432928</v>
       </c>
-      <c r="U20" t="inlineStr"/>
+      <c r="U20" s="2" t="n">
+        <v>429.7138297209178</v>
+      </c>
       <c r="V20" s="2" t="n">
-        <v>30.61949382134773</v>
+        <v>30.24186607511134</v>
       </c>
     </row>
     <row r="21">
@@ -7839,9 +8113,11 @@
       <c r="T21" s="2" t="n">
         <v>1026.949166151766</v>
       </c>
-      <c r="U21" t="inlineStr"/>
+      <c r="U21" s="2" t="n">
+        <v>19457.93966196803</v>
+      </c>
       <c r="V21" s="2" t="n">
-        <v>358.4885016531974</v>
+        <v>355.9925753030737</v>
       </c>
     </row>
     <row r="22">
@@ -7903,9 +8179,11 @@
       <c r="T22" s="2" t="n">
         <v>1402.543334729835</v>
       </c>
-      <c r="U22" t="inlineStr"/>
+      <c r="U22" s="2" t="n">
+        <v>36628.01043177136</v>
+      </c>
       <c r="V22" s="2" t="n">
-        <v>54263.25630566836</v>
+        <v>54468.06839372768</v>
       </c>
     </row>
     <row r="23">
@@ -7967,9 +8245,11 @@
       <c r="T23" s="2" t="n">
         <v>386.5475898419766</v>
       </c>
-      <c r="U23" t="inlineStr"/>
+      <c r="U23" s="2" t="n">
+        <v>7192.0799722064</v>
+      </c>
       <c r="V23" s="2" t="n">
-        <v>3599.433765358843</v>
+        <v>3756.974335796574</v>
       </c>
     </row>
     <row r="24">
@@ -8031,9 +8311,11 @@
       <c r="T24" s="2" t="n">
         <v>302.0977274593374</v>
       </c>
-      <c r="U24" t="inlineStr"/>
+      <c r="U24" s="2" t="n">
+        <v>6468.171903120117</v>
+      </c>
       <c r="V24" s="2" t="n">
-        <v>870.5705143647886</v>
+        <v>873.4544605300705</v>
       </c>
     </row>
     <row r="25">
@@ -8095,9 +8377,11 @@
       <c r="T25" s="2" t="n">
         <v>498.989545697963</v>
       </c>
-      <c r="U25" t="inlineStr"/>
+      <c r="U25" s="2" t="n">
+        <v>10482.76470212062</v>
+      </c>
       <c r="V25" s="2" t="n">
-        <v>1466.805513860761</v>
+        <v>1534.363238304007</v>
       </c>
     </row>
     <row r="26">
@@ -8159,9 +8443,11 @@
       <c r="T26" s="2" t="n">
         <v>365.7817877867718</v>
       </c>
-      <c r="U26" t="inlineStr"/>
+      <c r="U26" s="2" t="n">
+        <v>7302.41397314856</v>
+      </c>
       <c r="V26" s="2" t="n">
-        <v>2241.303470499185</v>
+        <v>2202.672861758966</v>
       </c>
     </row>
     <row r="27">
@@ -8223,9 +8509,11 @@
       <c r="T27" s="2" t="n">
         <v>214.8456254500286</v>
       </c>
-      <c r="U27" t="inlineStr"/>
+      <c r="U27" s="2" t="n">
+        <v>4639.367520250014</v>
+      </c>
       <c r="V27" s="2" t="n">
-        <v>914.7471558289719</v>
+        <v>912.4969484235231</v>
       </c>
     </row>
     <row r="28">
@@ -8287,9 +8575,11 @@
       <c r="T28" s="2" t="n">
         <v>58.57130611921327</v>
       </c>
-      <c r="U28" t="inlineStr"/>
+      <c r="U28" s="2" t="n">
+        <v>1241.732501053916</v>
+      </c>
       <c r="V28" s="2" t="n">
-        <v>51.47680407947213</v>
+        <v>52.04538846348984</v>
       </c>
     </row>
     <row r="29">
@@ -8351,9 +8641,11 @@
       <c r="T29" s="2" t="n">
         <v>33.96434110595385</v>
       </c>
-      <c r="U29" t="inlineStr"/>
+      <c r="U29" s="2" t="n">
+        <v>384.2199552505144</v>
+      </c>
       <c r="V29" s="2" t="n">
-        <v>15.84363644687813</v>
+        <v>15.74045856603944</v>
       </c>
     </row>
     <row r="30">
@@ -8415,9 +8707,11 @@
       <c r="T30" s="2" t="n">
         <v>238.5392806846162</v>
       </c>
-      <c r="U30" t="inlineStr"/>
+      <c r="U30" s="2" t="n">
+        <v>5890.540991774528</v>
+      </c>
       <c r="V30" s="2" t="n">
-        <v>973.8168227278527</v>
+        <v>1052.784035982254</v>
       </c>
     </row>
     <row r="31">
@@ -8479,9 +8773,11 @@
       <c r="T31" s="2" t="n">
         <v>124.4227433922786</v>
       </c>
-      <c r="U31" t="inlineStr"/>
+      <c r="U31" s="2" t="n">
+        <v>2077.93919423726</v>
+      </c>
       <c r="V31" s="2" t="n">
-        <v>257.2314406079555</v>
+        <v>264.6352371056698</v>
       </c>
     </row>
     <row r="32">
@@ -8543,9 +8839,11 @@
       <c r="T32" s="2" t="n">
         <v>62.51182103670719</v>
       </c>
-      <c r="U32" t="inlineStr"/>
+      <c r="U32" s="2" t="n">
+        <v>1076.569235856269</v>
+      </c>
       <c r="V32" s="2" t="n">
-        <v>49.44234709626252</v>
+        <v>49.22352449576737</v>
       </c>
     </row>
     <row r="33">
@@ -8607,9 +8905,11 @@
       <c r="T33" s="2" t="n">
         <v>79.06417419777897</v>
       </c>
-      <c r="U33" t="inlineStr"/>
+      <c r="U33" s="2" t="n">
+        <v>1336.899397230146</v>
+      </c>
       <c r="V33" s="2" t="n">
-        <v>55.21649223390927</v>
+        <v>54.37521282713333</v>
       </c>
     </row>
     <row r="34">
@@ -8671,7 +8971,9 @@
       <c r="T34" s="2" t="n">
         <v>93.93701586748909</v>
       </c>
-      <c r="U34" t="inlineStr"/>
+      <c r="U34" s="2" t="n">
+        <v>928.1296689436963</v>
+      </c>
       <c r="V34" s="2" t="n">
         <v>0</v>
       </c>
@@ -8735,9 +9037,11 @@
       <c r="T35" s="2" t="n">
         <v>37.34627814956497</v>
       </c>
-      <c r="U35" t="inlineStr"/>
+      <c r="U35" s="2" t="n">
+        <v>804.4519733709429</v>
+      </c>
       <c r="V35" s="2" t="n">
-        <v>434511.4558208574</v>
+        <v>432377.2805293642</v>
       </c>
     </row>
     <row r="36">
@@ -8799,9 +9103,11 @@
       <c r="T36" s="2" t="n">
         <v>49.63422125238045</v>
       </c>
-      <c r="U36" t="inlineStr"/>
+      <c r="U36" s="2" t="n">
+        <v>913.3481108780538</v>
+      </c>
       <c r="V36" s="2" t="n">
-        <v>34.58797955858259</v>
+        <v>34.44567748145593</v>
       </c>
     </row>
     <row r="37">
@@ -8863,9 +9169,11 @@
       <c r="T37" s="2" t="n">
         <v>20.15498389413338</v>
       </c>
-      <c r="U37" t="inlineStr"/>
+      <c r="U37" s="2" t="n">
+        <v>201.2434870999223</v>
+      </c>
       <c r="V37" s="2" t="n">
-        <v>6.806530774155014</v>
+        <v>6.798716360355339</v>
       </c>
     </row>
     <row r="38">
@@ -8927,9 +9235,11 @@
       <c r="T38" s="2" t="n">
         <v>13.40149257259501</v>
       </c>
-      <c r="U38" t="inlineStr"/>
+      <c r="U38" s="2" t="n">
+        <v>172.7076613488797</v>
+      </c>
       <c r="V38" s="2" t="n">
-        <v>6.748256808111043</v>
+        <v>6.701891479903765</v>
       </c>
     </row>
     <row r="39">
@@ -8991,9 +9301,11 @@
       <c r="T39" s="2" t="n">
         <v>38.31771921262021</v>
       </c>
-      <c r="U39" t="inlineStr"/>
+      <c r="U39" s="2" t="n">
+        <v>343.0664594737765</v>
+      </c>
       <c r="V39" s="2" t="n">
-        <v>7.614973097363993</v>
+        <v>7.435466290384134</v>
       </c>
     </row>
     <row r="40">
@@ -9055,7 +9367,9 @@
       <c r="T40" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="U40" t="inlineStr"/>
+      <c r="U40" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V40" s="2" t="n">
         <v>1</v>
       </c>
@@ -9119,7 +9433,9 @@
       <c r="T41" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="U41" t="inlineStr"/>
+      <c r="U41" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V41" s="2" t="n">
         <v>1</v>
       </c>
@@ -9331,7 +9647,9 @@
         <v>1</v>
       </c>
       <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V2" s="2" t="n">
         <v>1</v>
       </c>
@@ -9395,7 +9713,9 @@
       <c r="T3" s="2" t="n">
         <v>11.45573268643595</v>
       </c>
-      <c r="U3" t="inlineStr"/>
+      <c r="U3" s="2" t="n">
+        <v>96.79725031481013</v>
+      </c>
       <c r="V3" s="2" t="n">
         <v>0</v>
       </c>
@@ -9459,9 +9779,11 @@
       <c r="T4" s="2" t="n">
         <v>11.45573268643596</v>
       </c>
-      <c r="U4" t="inlineStr"/>
+      <c r="U4" s="2" t="n">
+        <v>31.99787761378754</v>
+      </c>
       <c r="V4" s="2" t="n">
-        <v>0.3042852088602726</v>
+        <v>0.3042852088602723</v>
       </c>
     </row>
     <row r="5">
@@ -9523,7 +9845,9 @@
       <c r="T5" s="2" t="n">
         <v>11.45573268643596</v>
       </c>
-      <c r="U5" t="inlineStr"/>
+      <c r="U5" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="V5" s="2" t="n">
         <v>0</v>
       </c>
@@ -9587,7 +9911,9 @@
       <c r="T6" s="2" t="n">
         <v>11.455732686436</v>
       </c>
-      <c r="U6" t="inlineStr"/>
+      <c r="U6" s="2" t="n">
+        <v>70.93194274175305</v>
+      </c>
       <c r="V6" s="2" t="n">
         <v>0</v>
       </c>
@@ -9651,7 +9977,9 @@
       <c r="T7" s="2" t="n">
         <v>589.4330104533043</v>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" s="2" t="n">
+        <v>16768.7649463136</v>
+      </c>
       <c r="V7" s="2" t="n">
         <v>0</v>
       </c>
@@ -9715,7 +10043,9 @@
       <c r="T8" s="2" t="n">
         <v>1159.573909469029</v>
       </c>
-      <c r="U8" t="inlineStr"/>
+      <c r="U8" s="2" t="n">
+        <v>16136.27866111681</v>
+      </c>
       <c r="V8" s="2" t="n">
         <v>0</v>
       </c>
@@ -9779,7 +10109,9 @@
       <c r="T9" s="2" t="n">
         <v>28472.38875010574</v>
       </c>
-      <c r="U9" t="inlineStr"/>
+      <c r="U9" s="2" t="n">
+        <v>738099.2528492853</v>
+      </c>
       <c r="V9" s="2" t="n">
         <v>0</v>
       </c>
@@ -9843,7 +10175,9 @@
       <c r="T10" s="2" t="n">
         <v>17716.55758727512</v>
       </c>
-      <c r="U10" t="inlineStr"/>
+      <c r="U10" s="2" t="n">
+        <v>336357.8280319945</v>
+      </c>
       <c r="V10" s="2" t="n">
         <v>0</v>
       </c>
@@ -9907,7 +10241,9 @@
       <c r="T11" s="2" t="n">
         <v>79829.74122683672</v>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" s="2" t="n">
+        <v>1740544.551125968</v>
+      </c>
       <c r="V11" s="2" t="n">
         <v>0</v>
       </c>
@@ -9971,9 +10307,11 @@
       <c r="T12" s="2" t="n">
         <v>1235.005059695206</v>
       </c>
-      <c r="U12" t="inlineStr"/>
+      <c r="U12" s="2" t="n">
+        <v>32229.81832902572</v>
+      </c>
       <c r="V12" s="2" t="n">
-        <v>8745.50225642875</v>
+        <v>9391.662138688902</v>
       </c>
     </row>
     <row r="13">
@@ -10035,9 +10373,11 @@
       <c r="T13" s="2" t="n">
         <v>625.6398525504122</v>
       </c>
-      <c r="U13" t="inlineStr"/>
+      <c r="U13" s="2" t="n">
+        <v>6535.006357642978</v>
+      </c>
       <c r="V13" s="2" t="n">
-        <v>84.84143089963365</v>
+        <v>84.26381301195687</v>
       </c>
     </row>
     <row r="14">
@@ -10099,9 +10439,11 @@
       <c r="T14" s="2" t="n">
         <v>136.6055189414853</v>
       </c>
-      <c r="U14" t="inlineStr"/>
+      <c r="U14" s="2" t="n">
+        <v>1664.508704060671</v>
+      </c>
       <c r="V14" s="2" t="n">
-        <v>124.5851469868333</v>
+        <v>126.7677064564085</v>
       </c>
     </row>
     <row r="15">
@@ -10163,9 +10505,11 @@
       <c r="T15" s="2" t="n">
         <v>549.444451049417</v>
       </c>
-      <c r="U15" t="inlineStr"/>
+      <c r="U15" s="2" t="n">
+        <v>8379.75005549382</v>
+      </c>
       <c r="V15" s="2" t="n">
-        <v>5737.693488981377</v>
+        <v>5872.867165714218</v>
       </c>
     </row>
     <row r="16">
@@ -10227,9 +10571,11 @@
       <c r="T16" s="2" t="n">
         <v>495.1925234658902</v>
       </c>
-      <c r="U16" t="inlineStr"/>
+      <c r="U16" s="2" t="n">
+        <v>4943.256155546237</v>
+      </c>
       <c r="V16" s="2" t="n">
-        <v>97.89018675463855</v>
+        <v>95.42795852018388</v>
       </c>
     </row>
     <row r="17">
@@ -10291,9 +10637,11 @@
       <c r="T17" s="2" t="n">
         <v>1638.427424642126</v>
       </c>
-      <c r="U17" t="inlineStr"/>
+      <c r="U17" s="2" t="n">
+        <v>28224.76191993072</v>
+      </c>
       <c r="V17" s="2" t="n">
-        <v>501070.8445438638</v>
+        <v>528322.7833985733</v>
       </c>
     </row>
     <row r="18">
@@ -10355,9 +10703,11 @@
       <c r="T18" s="2" t="n">
         <v>173.9685924898981</v>
       </c>
-      <c r="U18" t="inlineStr"/>
+      <c r="U18" s="2" t="n">
+        <v>2138.179836778507</v>
+      </c>
       <c r="V18" s="2" t="n">
-        <v>365808.4816779341</v>
+        <v>368059.0505787696</v>
       </c>
     </row>
     <row r="19">
@@ -10419,9 +10769,11 @@
       <c r="T19" s="2" t="n">
         <v>673.4293131078545</v>
       </c>
-      <c r="U19" t="inlineStr"/>
+      <c r="U19" s="2" t="n">
+        <v>8955.769671676242</v>
+      </c>
       <c r="V19" s="2" t="n">
-        <v>9104.502390041736</v>
+        <v>9372.190554609972</v>
       </c>
     </row>
     <row r="20">
@@ -10483,9 +10835,11 @@
       <c r="T20" s="2" t="n">
         <v>31.78984884432919</v>
       </c>
-      <c r="U20" t="inlineStr"/>
+      <c r="U20" s="2" t="n">
+        <v>429.7138297209178</v>
+      </c>
       <c r="V20" s="2" t="n">
-        <v>30.61949382134773</v>
+        <v>30.24186607511134</v>
       </c>
     </row>
     <row r="21">
@@ -10547,9 +10901,11 @@
       <c r="T21" s="2" t="n">
         <v>1204.59770274904</v>
       </c>
-      <c r="U21" t="inlineStr"/>
+      <c r="U21" s="2" t="n">
+        <v>19477.73428974959</v>
+      </c>
       <c r="V21" s="2" t="n">
-        <v>405.7311300126785</v>
+        <v>404.581424731353</v>
       </c>
     </row>
     <row r="22">
@@ -10611,9 +10967,11 @@
       <c r="T22" s="2" t="n">
         <v>1541.376378024101</v>
       </c>
-      <c r="U22" t="inlineStr"/>
+      <c r="U22" s="2" t="n">
+        <v>36646.10699017055</v>
+      </c>
       <c r="V22" s="2" t="n">
-        <v>54323.49203517471</v>
+        <v>54529.85719269228</v>
       </c>
     </row>
     <row r="23">
@@ -10675,9 +11033,11 @@
       <c r="T23" s="2" t="n">
         <v>402.7419296743773</v>
       </c>
-      <c r="U23" t="inlineStr"/>
+      <c r="U23" s="2" t="n">
+        <v>7193.837765876404</v>
+      </c>
       <c r="V23" s="2" t="n">
-        <v>3637.910840168317</v>
+        <v>3797.612340999315</v>
       </c>
     </row>
     <row r="24">
@@ -10739,9 +11099,11 @@
       <c r="T24" s="2" t="n">
         <v>320.873839433629</v>
       </c>
-      <c r="U24" t="inlineStr"/>
+      <c r="U24" s="2" t="n">
+        <v>6470.309337943433</v>
+      </c>
       <c r="V24" s="2" t="n">
-        <v>877.1168870485229</v>
+        <v>879.9238041237845</v>
       </c>
     </row>
     <row r="25">
@@ -10803,9 +11165,11 @@
       <c r="T25" s="2" t="n">
         <v>503.8815306468321</v>
       </c>
-      <c r="U25" t="inlineStr"/>
+      <c r="U25" s="2" t="n">
+        <v>10483.56369063844</v>
+      </c>
       <c r="V25" s="2" t="n">
-        <v>1469.329582827618</v>
+        <v>1536.980813788296</v>
       </c>
     </row>
     <row r="26">
@@ -10867,9 +11231,11 @@
       <c r="T26" s="2" t="n">
         <v>369.116222572059</v>
       </c>
-      <c r="U26" t="inlineStr"/>
+      <c r="U26" s="2" t="n">
+        <v>7302.838698035887</v>
+      </c>
       <c r="V26" s="2" t="n">
-        <v>2244.781283997163</v>
+        <v>2206.173007621883</v>
       </c>
     </row>
     <row r="27">
@@ -10931,9 +11297,11 @@
       <c r="T27" s="2" t="n">
         <v>217.2875903163548</v>
       </c>
-      <c r="U27" t="inlineStr"/>
+      <c r="U27" s="2" t="n">
+        <v>4639.642195872154</v>
+      </c>
       <c r="V27" s="2" t="n">
-        <v>916.7013995854682</v>
+        <v>914.4877172888382</v>
       </c>
     </row>
     <row r="28">
@@ -10995,9 +11363,11 @@
       <c r="T28" s="2" t="n">
         <v>61.65400644127671</v>
       </c>
-      <c r="U28" t="inlineStr"/>
+      <c r="U28" s="2" t="n">
+        <v>1242.265248765626</v>
+      </c>
       <c r="V28" s="2" t="n">
-        <v>52.02426211536708</v>
+        <v>52.60220453997403</v>
       </c>
     </row>
     <row r="29">
@@ -11059,9 +11429,11 @@
       <c r="T29" s="2" t="n">
         <v>37.73815678440172</v>
       </c>
-      <c r="U29" t="inlineStr"/>
+      <c r="U29" s="2" t="n">
+        <v>384.4560615417278</v>
+      </c>
       <c r="V29" s="2" t="n">
-        <v>16.09268302089474</v>
+        <v>15.98764928155265</v>
       </c>
     </row>
     <row r="30">
@@ -11123,9 +11495,11 @@
       <c r="T30" s="2" t="n">
         <v>241.8699624447206</v>
       </c>
-      <c r="U30" t="inlineStr"/>
+      <c r="U30" s="2" t="n">
+        <v>5891.013992800264</v>
+      </c>
       <c r="V30" s="2" t="n">
-        <v>975.6572812760189</v>
+        <v>1054.680271904452</v>
       </c>
     </row>
     <row r="31">
@@ -11187,9 +11561,11 @@
       <c r="T31" s="2" t="n">
         <v>124.422743392304</v>
       </c>
-      <c r="U31" t="inlineStr"/>
+      <c r="U31" s="2" t="n">
+        <v>2077.93919423726</v>
+      </c>
       <c r="V31" s="2" t="n">
-        <v>257.2314406079555</v>
+        <v>264.6352371056698</v>
       </c>
     </row>
     <row r="32">
@@ -11251,9 +11627,11 @@
       <c r="T32" s="2" t="n">
         <v>62.51182105004475</v>
       </c>
-      <c r="U32" t="inlineStr"/>
+      <c r="U32" s="2" t="n">
+        <v>1076.569235856269</v>
+      </c>
       <c r="V32" s="2" t="n">
-        <v>49.44234709626252</v>
+        <v>49.22352449576737</v>
       </c>
     </row>
     <row r="33">
@@ -11315,9 +11693,11 @@
       <c r="T33" s="2" t="n">
         <v>79.06417419779746</v>
       </c>
-      <c r="U33" t="inlineStr"/>
+      <c r="U33" s="2" t="n">
+        <v>1336.899397230146</v>
+      </c>
       <c r="V33" s="2" t="n">
-        <v>55.21649223390927</v>
+        <v>54.37521282713333</v>
       </c>
     </row>
     <row r="34">
@@ -11379,9 +11759,11 @@
       <c r="T34" s="2" t="n">
         <v>116.6919459632657</v>
       </c>
-      <c r="U34" t="inlineStr"/>
+      <c r="U34" s="2" t="n">
+        <v>929.6229819684345</v>
+      </c>
       <c r="V34" s="2" t="n">
-        <v>3.014062032192841</v>
+        <v>3.093012786806117</v>
       </c>
     </row>
     <row r="35">
@@ -11443,9 +11825,11 @@
       <c r="T35" s="2" t="n">
         <v>37.34627814956625</v>
       </c>
-      <c r="U35" t="inlineStr"/>
+      <c r="U35" s="2" t="n">
+        <v>804.4519733709429</v>
+      </c>
       <c r="V35" s="2" t="n">
-        <v>434511.4558208574</v>
+        <v>432377.2805293642</v>
       </c>
     </row>
     <row r="36">
@@ -11507,9 +11891,11 @@
       <c r="T36" s="2" t="n">
         <v>49.63422125238241</v>
       </c>
-      <c r="U36" t="inlineStr"/>
+      <c r="U36" s="2" t="n">
+        <v>913.3481108780538</v>
+      </c>
       <c r="V36" s="2" t="n">
-        <v>34.58797955858259</v>
+        <v>34.44567748145593</v>
       </c>
     </row>
     <row r="37">
@@ -11571,9 +11957,11 @@
       <c r="T37" s="2" t="n">
         <v>20.1549838941379</v>
       </c>
-      <c r="U37" t="inlineStr"/>
+      <c r="U37" s="2" t="n">
+        <v>201.2434870999223</v>
+      </c>
       <c r="V37" s="2" t="n">
-        <v>6.806530774155014</v>
+        <v>6.798716360355339</v>
       </c>
     </row>
     <row r="38">
@@ -11635,9 +12023,11 @@
       <c r="T38" s="2" t="n">
         <v>13.40149257259495</v>
       </c>
-      <c r="U38" t="inlineStr"/>
+      <c r="U38" s="2" t="n">
+        <v>172.7076613488797</v>
+      </c>
       <c r="V38" s="2" t="n">
-        <v>6.748256808111043</v>
+        <v>6.701891479903765</v>
       </c>
     </row>
     <row r="39">
@@ -11699,9 +12089,11 @@
       <c r="T39" s="2" t="n">
         <v>38.31771921262021</v>
       </c>
-      <c r="U39" t="inlineStr"/>
+      <c r="U39" s="2" t="n">
+        <v>343.0664594737765</v>
+      </c>
       <c r="V39" s="2" t="n">
-        <v>7.614973097363993</v>
+        <v>7.435466290384134</v>
       </c>
     </row>
     <row r="40">
@@ -11763,7 +12155,9 @@
       <c r="T40" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="U40" t="inlineStr"/>
+      <c r="U40" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V40" s="2" t="n">
         <v>1</v>
       </c>
@@ -11827,7 +12221,9 @@
       <c r="T41" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="U41" t="inlineStr"/>
+      <c r="U41" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="V41" s="2" t="n">
         <v>1</v>
       </c>
@@ -13302,22 +13698,22 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>0</v>
+        <v>66472.83403682434</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0</v>
+        <v>66462.18629421291</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>0</v>
+        <v>1378.874116073328</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>11273.05644750595</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>0</v>
+        <v>5.895666947442368</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>0</v>
+        <v>0.1223159062933984</v>
       </c>
     </row>
     <row r="21">
@@ -13327,22 +13723,22 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>10026.22286351984</v>
+        <v>10064.06728186468</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>9989.881880885045</v>
+        <v>10027.19170922459</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>9989.881880885045</v>
+        <v>10027.19170922459</v>
       </c>
       <c r="E21" s="2" t="n">
         <v>11273.05644750595</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>0.8861733219738471</v>
+        <v>0.8894829681654792</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>0.8861733219738471</v>
+        <v>0.8894829681654792</v>
       </c>
     </row>
   </sheetData>
@@ -13418,25 +13814,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>75</v>
+        <v>98</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
     </row>
     <row r="3">
@@ -13446,10 +13842,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C3" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -13645,7 +14041,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Christensen &amp; Pauly (1995): per-group TE^(1-TL) with global_TE=0.1.</t>
+          <t>Pauly &amp; Christensen (1995): per-group TE^(1-TL) with global_TE=0.1.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -13662,7 +14058,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Christensen &amp; Pauly (1995): per-group TE^(1-TL) with global_TE='mean'.</t>
+          <t>Pauly &amp; Christensen (1995): per-group TE^(1-TL) with global_TE='mean'.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">

</xml_diff>